<commit_message>
fix(sami): extend v2 fixture and add Survey Completed to RESPONSES_OPTIONAL
The real export has 39 columns; the fixture had only 31. Added the 8 missing
columns (City Location, Destination_other, Prev_country_other, Re-engagement Sent At,
Survey Completed, Survey Sent, origin_country, transit) to fixture and extended
all row tuples to match. Survey Completed is now RESPONSES_OPTIONAL, not IGNORED,
since it is genuinely useful for survey response-rate analysis.

Both real export and fixture now produce zero unknown column warnings.
</commit_message>
<xml_diff>
--- a/tests/fixtures/users_v2.xlsx
+++ b/tests/fixtures/users_v2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AM10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,6 +584,46 @@
       <c r="AE3" t="inlineStr">
         <is>
           <t>Migrated From v1</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>City Location</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Destination_other</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Prev_country_other</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Re-engagement Sent At</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Survey Completed</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>Survey Sent</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>origin_country</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>transit</t>
         </is>
       </c>
     </row>

</xml_diff>